<commit_message>
Harden affection plan agent workflow
</commit_message>
<xml_diff>
--- a/data/siteplan.xlsx
+++ b/data/siteplan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zulfiqar/Documents/IMKANProjects/apps/ai-automation-agent/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FCFCDF8-3150-7142-AC54-7107963963CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B42EA46-3123-214D-ACB9-7CF1BEDF9B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16640" yWindow="6480" windowWidth="34560" windowHeight="21660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Site Plans" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="4">
   <si>
     <t>Unit Name</t>
   </si>
@@ -31,29 +31,14 @@
     <t>Plot Number</t>
   </si>
   <si>
-    <t>Villa 1</t>
-  </si>
-  <si>
     <t>Type A</t>
-  </si>
-  <si>
-    <t>Villa 2</t>
-  </si>
-  <si>
-    <t>PS4</t>
-  </si>
-  <si>
-    <t>SS18</t>
-  </si>
-  <si>
-    <t>P127</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -66,6 +51,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="2">
@@ -88,8 +78,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,7 +420,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -444,41 +435,350 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>3</v>
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1187</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1188</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1189</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1190</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1223</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1230</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1348</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9">
         <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1237</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1246</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" s="1">
+        <v>1328</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="1">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="1">
+        <v>1317</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="1">
+        <v>1318</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1319</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1320</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="1">
+        <v>1280</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="1">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1282</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>3</v>
+      </c>
+      <c r="C21" s="1">
+        <v>1315</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22" s="1">
+        <v>1316</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="1">
+        <v>1314</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>3</v>
+      </c>
+      <c r="C24" s="1">
+        <v>1313</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>3</v>
+      </c>
+      <c r="C25" s="1">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26" s="1">
+        <v>1311</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>3</v>
+      </c>
+      <c r="C27" s="1">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>3</v>
+      </c>
+      <c r="C28" s="1">
+        <v>1306</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>3</v>
+      </c>
+      <c r="C29" s="1">
+        <v>1305</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>3</v>
+      </c>
+      <c r="C30" s="1">
+        <v>1296</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>3</v>
+      </c>
+      <c r="C31" s="1">
+        <v>1297</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>3</v>
+      </c>
+      <c r="C32" s="1">
+        <v>1357</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <ignoredErrors>
     <ignoredError sqref="A1:C1" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>